<commit_message>
rerun all modules with updated cpg list
</commit_message>
<xml_diff>
--- a/analyses/demo-clin-stats/results/demo-clin-pvalues-by-histology.xlsx
+++ b/analyses/demo-clin-stats/results/demo-clin-pvalues-by-histology.xlsx
@@ -398,7 +398,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.258370854717028</v>
+        <v>0.208898590097032</v>
       </c>
     </row>
     <row r="3">
@@ -406,7 +406,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>0.1408182448886</v>
+        <v>0.181379191028179</v>
       </c>
     </row>
     <row r="4">
@@ -414,7 +414,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>0.830977487111851</v>
+        <v>0.879822457370452</v>
       </c>
     </row>
     <row r="5">
@@ -422,7 +422,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.661238327317944</v>
+        <v>0.989583655271352</v>
       </c>
     </row>
     <row r="6">
@@ -430,7 +430,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>0.143818354993677</v>
+        <v>0.150730466080972</v>
       </c>
     </row>
     <row r="7">
@@ -438,7 +438,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>0.868300106934329</v>
+        <v>0.899590041661931</v>
       </c>
     </row>
     <row r="8">
@@ -446,7 +446,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.148440568057781</v>
+        <v>0.0887794516423712</v>
       </c>
     </row>
     <row r="9">
@@ -813,7 +813,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.33006993006993</v>
+        <v>0.468531468531469</v>
       </c>
     </row>
     <row r="3">
@@ -821,7 +821,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>0.230769230769231</v>
       </c>
     </row>
     <row r="4">
@@ -829,7 +829,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>0.664335664335665</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -837,7 +837,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.328671328671329</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -853,7 +853,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>0.111111111111111</v>
+        <v>0.222222222222222</v>
       </c>
     </row>
     <row r="8">
@@ -861,7 +861,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.666666666666667</v>
+        <v>0.222222222222222</v>
       </c>
     </row>
     <row r="9">
@@ -1062,7 +1062,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.099269066823374</v>
+        <v>0.0608967811643551</v>
       </c>
     </row>
     <row r="3">
@@ -1070,7 +1070,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>0.647110170368091</v>
+        <v>0.490758227237542</v>
       </c>
     </row>
     <row r="4">
@@ -1078,7 +1078,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>0.976232230683878</v>
+        <v>0.946079289753066</v>
       </c>
     </row>
     <row r="5">
@@ -1086,7 +1086,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.950212628821588</v>
+        <v>0.971915975844798</v>
       </c>
     </row>
     <row r="6">
@@ -1094,7 +1094,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>0.410362840774718</v>
+        <v>0.399888854575204</v>
       </c>
     </row>
     <row r="7">
@@ -1102,7 +1102,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>0.00307470546413358</v>
+        <v>0.00146642909604224</v>
       </c>
     </row>
     <row r="8">
@@ -1110,7 +1110,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.00261898965050277</v>
+        <v>0.000562193700528096</v>
       </c>
     </row>
     <row r="9">
@@ -1228,7 +1228,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.106717016062028</v>
+        <v>0.179338963202914</v>
       </c>
     </row>
     <row r="3">
@@ -1236,7 +1236,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>0.765661101678121</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1244,7 +1244,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>0.474483025747333</v>
+        <v>0.790277848812941</v>
       </c>
     </row>
     <row r="5">
@@ -1252,7 +1252,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.293332234357925</v>
+        <v>0.508479501999196</v>
       </c>
     </row>
     <row r="6">
@@ -1268,7 +1268,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>0.194785106832606</v>
+        <v>0.0746960852443792</v>
       </c>
     </row>
     <row r="8">
@@ -1276,7 +1276,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.0979396497170013</v>
+        <v>0.0206858917243287</v>
       </c>
     </row>
     <row r="9">
@@ -1311,7 +1311,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.19955781429289</v>
+        <v>0.35853840492135</v>
       </c>
     </row>
     <row r="3">
@@ -1319,7 +1319,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>0.309865431987481</v>
+        <v>0.282490145116547</v>
       </c>
     </row>
     <row r="4">
@@ -1327,7 +1327,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>0.248632198653321</v>
+        <v>0.195050673701128</v>
       </c>
     </row>
     <row r="5">
@@ -1343,7 +1343,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>0.276011201785736</v>
+        <v>0.229633229215357</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
update sex for Tables 1, S9
</commit_message>
<xml_diff>
--- a/analyses/demo-clin-stats/results/demo-clin-pvalues-by-histology.xlsx
+++ b/analyses/demo-clin-stats/results/demo-clin-pvalues-by-histology.xlsx
@@ -1319,7 +1319,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>0.282490145116547</v>
+        <v>0.809253080892281</v>
       </c>
     </row>
     <row r="4">
@@ -1335,7 +1335,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.0735420797512746</v>
+        <v>0.00189775351983205</v>
       </c>
     </row>
     <row r="6">
@@ -1651,7 +1651,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>0.760344776517266</v>
+        <v>0.671061457964899</v>
       </c>
     </row>
     <row r="4">
@@ -1667,7 +1667,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.870022337929905</v>
+        <v>0.557245481646934</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
rerun demo clin stats module
</commit_message>
<xml_diff>
--- a/analyses/demo-clin-stats/results/demo-clin-pvalues-by-histology.xlsx
+++ b/analyses/demo-clin-stats/results/demo-clin-pvalues-by-histology.xlsx
@@ -1319,7 +1319,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>0.809253080892281</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1651,7 +1651,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>0.671061457964899</v>
+        <v>0.683396653291215</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
use germline sex estimate in demo clin stats
</commit_message>
<xml_diff>
--- a/analyses/demo-clin-stats/results/demo-clin-pvalues-by-histology.xlsx
+++ b/analyses/demo-clin-stats/results/demo-clin-pvalues-by-histology.xlsx
@@ -398,7 +398,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.208898590097032</v>
+        <v>0.141406276878222</v>
       </c>
     </row>
     <row r="3">
@@ -406,7 +406,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>0.181379191028179</v>
+        <v>0.187602210449896</v>
       </c>
     </row>
     <row r="4">
@@ -414,7 +414,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>0.879822457370452</v>
+        <v>0.787210041469433</v>
       </c>
     </row>
     <row r="5">
@@ -422,7 +422,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.989583655271352</v>
+        <v>0.629239390426486</v>
       </c>
     </row>
     <row r="6">
@@ -430,7 +430,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>0.150730466080972</v>
+        <v>0.0658497860932072</v>
       </c>
     </row>
     <row r="7">
@@ -438,7 +438,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>0.899590041661931</v>
+        <v>0.780960616370601</v>
       </c>
     </row>
     <row r="8">
@@ -446,7 +446,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.0887794516423712</v>
+        <v>0.050344850077476</v>
       </c>
     </row>
     <row r="9">
@@ -813,7 +813,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.468531468531469</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -821,7 +821,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>0.230769230769231</v>
+        <v>0.104895104895105</v>
       </c>
     </row>
     <row r="4">
@@ -829,7 +829,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>0.664335664335665</v>
       </c>
     </row>
     <row r="5">
@@ -837,7 +837,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0.328671328671329</v>
       </c>
     </row>
     <row r="6">
@@ -853,7 +853,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>0.222222222222222</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -861,7 +861,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.222222222222222</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1062,7 +1062,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0608967811643551</v>
+        <v>0.0402240016088645</v>
       </c>
     </row>
     <row r="3">
@@ -1070,7 +1070,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>0.490758227237542</v>
+        <v>0.359603620528773</v>
       </c>
     </row>
     <row r="4">
@@ -1078,7 +1078,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>0.946079289753066</v>
+        <v>0.976232230683878</v>
       </c>
     </row>
     <row r="5">
@@ -1086,7 +1086,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.971915975844798</v>
+        <v>0.950212628821588</v>
       </c>
     </row>
     <row r="6">
@@ -1094,7 +1094,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>0.399888854575204</v>
+        <v>0.410362840774718</v>
       </c>
     </row>
     <row r="7">
@@ -1102,7 +1102,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>0.00146642909604224</v>
+        <v>0.00360183991293667</v>
       </c>
     </row>
     <row r="8">
@@ -1110,7 +1110,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.000562193700528096</v>
+        <v>0.00149243163401454</v>
       </c>
     </row>
     <row r="9">
@@ -1319,7 +1319,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>0.012349824785448</v>
       </c>
     </row>
     <row r="4">
@@ -1335,7 +1335,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.00189775351983205</v>
+        <v>0.0735420797512746</v>
       </c>
     </row>
     <row r="6">
@@ -1643,7 +1643,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.285789423282333</v>
+        <v>0.737683929945924</v>
       </c>
     </row>
     <row r="3">
@@ -1651,7 +1651,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>0.683396653291215</v>
+        <v>0.257876928370706</v>
       </c>
     </row>
     <row r="4">
@@ -1659,7 +1659,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>0.999999999999994</v>
+        <v>0.623933115738392</v>
       </c>
     </row>
     <row r="5">
@@ -1667,7 +1667,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.557245481646934</v>
+        <v>0.514027191184935</v>
       </c>
     </row>
     <row r="6">
@@ -1675,7 +1675,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>0.999999999999997</v>
+        <v>0.875037840336952</v>
       </c>
     </row>
     <row r="7">
@@ -1683,7 +1683,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>0.4606509551112</v>
+        <v>0.817856208885551</v>
       </c>
     </row>
     <row r="8">
@@ -1691,7 +1691,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.291184371184371</v>
+        <v>0.764245899028508</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
rm unk sex from fisher test
</commit_message>
<xml_diff>
--- a/analyses/demo-clin-stats/results/demo-clin-pvalues-by-histology.xlsx
+++ b/analyses/demo-clin-stats/results/demo-clin-pvalues-by-histology.xlsx
@@ -1319,7 +1319,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>0.012349824785448</v>
+        <v>0.560817490737391</v>
       </c>
     </row>
     <row r="4">
@@ -1651,7 +1651,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>0.257876928370706</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">

</xml_diff>